<commit_message>
6.OG: čisté podklady pro MH BIM (osa 39×E jako počátek), ořez --oblast, oprava purge bloků kót
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NLNxwuW9bh8oL1SbiMzDu4
</commit_message>
<xml_diff>
--- a/vystupy/MHBIM_zadavaci_list.xlsx
+++ b/vystupy/MHBIM_zadavaci_list.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Vztažný bod = průsečík os / roh nosné konstrukce, který je ve všech podlažích. Sozialgebäude má jiný souřadný systém (X≈-1,5 mil.) – posun nutný.</t>
+          <t>Vztažný bod = průsečík osy 39 a osy E (v 6.OG X=24331, Y=68325). Ověřit, že ostatní podlaží mají stejnou osovou síť a souřadnice. Sozialgebäude má jiný souřadný systém (X≈-1,5 mil.) – posun nutný.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -809,7 +809,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Podklad vložen v MH BIM</t>
+          <t>Čistý podklad / vložen v MH BIM</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -1036,8 +1036,16 @@
         <v>5000</v>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>24331,68325 (osa 39 × E)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>podklad hotov: vystupy/podklady_mhbim/6OG_*.dxf</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Versorgungsgang: čisté podklady (DWG z Drive přes LibreDWG), vztažný bod po podlažích, oprava DXF z dwg2dxf
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NLNxwuW9bh8oL1SbiMzDu4
</commit_message>
<xml_diff>
--- a/vystupy/MHBIM_zadavaci_list.xlsx
+++ b/vystupy/MHBIM_zadavaci_list.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Vztažný bod = průsečík osy 39 a osy E (v 6.OG X=24331, Y=68325). Ověřit, že ostatní podlaží mají stejnou osovou síť a souřadnice. Sozialgebäude má jiný souřadný systém (X≈-1,5 mil.) – posun nutný.</t>
+          <t>Vztažný bod = průsečík osy 39 a osy E – KAŽDÉ podlaží má jiné souřadnice (6.OG 24331,68325; Versorgungsgang 20618,69827), zjistit pro každé zvlášť. Sozialgebäude má jiný souřadný systém (X≈-1,5 mil.) – posun nutný.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -1098,8 +1098,16 @@
         <v>2700</v>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>20618,69827 (osa 39 × E)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>podklad hotov: vystupy/podklady_mhbim/Versorgungsgang_*.dxf</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>